<commit_message>
feat: quality vocab, KPI dashboard, traps, and English doc tree cleanup
Land concurrent work (quality layer-2, KPI panel, format variants, traps) on the
rewritten English documentation history, drop timeline/handoff by choice, and
renumber benchmarks/system docs accordingly.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/synthetic/MTO_sugerencias.xlsx
+++ b/data/synthetic/MTO_sugerencias.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="175">
   <si>
     <t>MTO SINTÉTICO — un token por columna, para imputar varios vocabularios</t>
   </si>
@@ -110,15 +110,111 @@
     <t>niquelado</t>
   </si>
   <si>
+    <t>M12x40</t>
+  </si>
+  <si>
+    <t>HDG</t>
+  </si>
+  <si>
+    <t>M14x50</t>
+  </si>
+  <si>
+    <t>GALVA</t>
+  </si>
+  <si>
+    <t>M10x35</t>
+  </si>
+  <si>
+    <t>YZP</t>
+  </si>
+  <si>
+    <t>Vis</t>
+  </si>
+  <si>
+    <t>M10x45</t>
+  </si>
+  <si>
+    <t>ISO 4017</t>
+  </si>
+  <si>
+    <t>zingue</t>
+  </si>
+  <si>
+    <t>M8x25</t>
+  </si>
+  <si>
+    <t>black</t>
+  </si>
+  <si>
+    <t>M16x50</t>
+  </si>
+  <si>
+    <t>phosphate</t>
+  </si>
+  <si>
+    <t>Tuerca</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>M10</t>
+  </si>
+  <si>
+    <t>DIN 934</t>
+  </si>
+  <si>
+    <t>zincadas</t>
+  </si>
+  <si>
+    <t>M12x60</t>
+  </si>
+  <si>
+    <t>Ruspert 1000</t>
+  </si>
+  <si>
+    <t>M16x80</t>
+  </si>
+  <si>
+    <t>Geomet 500</t>
+  </si>
+  <si>
+    <t>M20x70</t>
+  </si>
+  <si>
+    <t>Dacromet 320</t>
+  </si>
+  <si>
+    <t>M24x100</t>
+  </si>
+  <si>
+    <t>sherardizado</t>
+  </si>
+  <si>
+    <t>M10x50</t>
+  </si>
+  <si>
+    <t>zinc-niquel</t>
+  </si>
+  <si>
+    <t>M12x30</t>
+  </si>
+  <si>
+    <t>galv</t>
+  </si>
+  <si>
+    <t>M8x20</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
     <t>Espárrago</t>
   </si>
   <si>
     <t>GR L7</t>
   </si>
   <si>
-    <t>M8x20</t>
-  </si>
-  <si>
     <t>ASTM A320</t>
   </si>
   <si>
@@ -128,18 +224,12 @@
     <t>GR B8</t>
   </si>
   <si>
-    <t>M16x80</t>
-  </si>
-  <si>
     <t>ASTM A193</t>
   </si>
   <si>
     <t>geomet</t>
   </si>
   <si>
-    <t>Tuerca</t>
-  </si>
-  <si>
     <t>GR 12H</t>
   </si>
   <si>
@@ -149,6 +239,57 @@
     <t>ISO 4032</t>
   </si>
   <si>
+    <t>GR B16</t>
+  </si>
+  <si>
+    <t>M20x100</t>
+  </si>
+  <si>
+    <t>A4-80</t>
+  </si>
+  <si>
+    <t>GRADE 5</t>
+  </si>
+  <si>
+    <t>M12x45</t>
+  </si>
+  <si>
+    <t>A2-80</t>
+  </si>
+  <si>
+    <t>M6x20</t>
+  </si>
+  <si>
+    <t>GR B8M</t>
+  </si>
+  <si>
+    <t>M12x70</t>
+  </si>
+  <si>
+    <t>GR 660</t>
+  </si>
+  <si>
+    <t>M16x90</t>
+  </si>
+  <si>
+    <t>ASTM A453</t>
+  </si>
+  <si>
+    <t>Arandela</t>
+  </si>
+  <si>
+    <t>200HV</t>
+  </si>
+  <si>
+    <t>M16</t>
+  </si>
+  <si>
+    <t>DIN 125</t>
+  </si>
+  <si>
+    <t>zincada</t>
+  </si>
+  <si>
     <t>vis</t>
   </si>
   <si>
@@ -161,21 +302,51 @@
     <t>UNI 5737</t>
   </si>
   <si>
+    <t>Schraube</t>
+  </si>
+  <si>
+    <t>verzinkt</t>
+  </si>
+  <si>
+    <t>M6x16</t>
+  </si>
+  <si>
+    <t>parafuso</t>
+  </si>
+  <si>
     <t>M16x70</t>
   </si>
   <si>
     <t>WN 70</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>M20</t>
   </si>
   <si>
     <t>ASME B18.2.2</t>
   </si>
   <si>
+    <t>M16x55</t>
+  </si>
+  <si>
+    <t>UNI 5739</t>
+  </si>
+  <si>
+    <t>GR R</t>
+  </si>
+  <si>
+    <t>M20x65</t>
+  </si>
+  <si>
+    <t>BS 3692</t>
+  </si>
+  <si>
+    <t>galvanizado en caliente</t>
+  </si>
+  <si>
+    <t>M20x110</t>
+  </si>
+  <si>
     <t>GR L43</t>
   </si>
   <si>
@@ -185,9 +356,6 @@
     <t>A4-70</t>
   </si>
   <si>
-    <t>DIN 934</t>
-  </si>
-  <si>
     <t>VOCABULARIO</t>
   </si>
   <si>
@@ -227,6 +395,54 @@
     <t>acabado "niquelado" → 8º acabado: escalar / no es acabado (no autoservicio)</t>
   </si>
   <si>
+    <t>control</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>control: "HDG" ya es alias de GALVANIZADO EN CALIENTE → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>control: "GALVA" ya es alias de GALVANIZADO EN CALIENTE → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>control: "YZP" ya es alias de BICROMATADO → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>control: "zingue" (FR) ya es alias de CINCADO, acento plegado → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>control: "black" ya es alias de PAVONADO → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>control: "phosphate" ya es alias de FOSFATADO → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>control: "zincadas" (concordancia) ya es alias de CINCADO → resuelta por tabla</t>
+  </si>
+  <si>
+    <t>acabado "Ruspert 1000" → candidato a alias de GEOMET (o escalar si el cliente lo separa)</t>
+  </si>
+  <si>
+    <t>acabado "Geomet 500" → candidato a alias de GEOMET</t>
+  </si>
+  <si>
+    <t>acabado "Dacromet 320" → candidato a alias de DACROMET</t>
+  </si>
+  <si>
+    <t>acabado "sherardizado" → no es ninguno de los 7 de §9: escalar, NO autoservicio</t>
+  </si>
+  <si>
+    <t>acabado "zinc-niquel" → aleación, fuera de §9: escalar, NO autoservicio</t>
+  </si>
+  <si>
+    <t>acabado "galv" a secas → ambiguo entre CINCADO y GALVANIZADO EN CALIENTE: el alta la decide el cliente, no nosotros</t>
+  </si>
+  <si>
+    <t>acabado "A2" → es una calidad de §5, no un acabado: la guarda entre atributos aún no existe (07-solucion-objetivo, línea 5); hoy se dejaría dar de alta</t>
+  </si>
+  <si>
     <t>material</t>
   </si>
   <si>
@@ -242,7 +458,28 @@
     <t>no (solo lectura)</t>
   </si>
   <si>
-    <t>calidad "GR 12H" fuera de §5 (45H ya está decidida) → hueco de calidad; calidad es solo lectura hoy</t>
+    <t>calidad "GR 12H" fuera de §5 (45H ya está decidida) → hueco de calidad con candidata; alta ágil en /vocabulario?attr=quality eligiendo grupo (SPEC-016)</t>
+  </si>
+  <si>
+    <t>control: "GR B16" tiene entrada en la tabla → material AC sin tocar nada</t>
+  </si>
+  <si>
+    <t>control: "A4-80" es G4 → INOX por tabla; y G4 no se convierte a G3 (A4)</t>
+  </si>
+  <si>
+    <t>control: "GRADE 5" es G5 → AC por tabla</t>
+  </si>
+  <si>
+    <t>control: "A2-80" es G2 AISLADO → INOX por tabla, y NO equivale a A2</t>
+  </si>
+  <si>
+    <t>calidad "GR B8M" (A193 inox con molibdeno) sin entrada → hueco P-3 con candidata INOX</t>
+  </si>
+  <si>
+    <t>calidad "GR 660" (A453, superaleación) sin entrada → hueco P-3; no se deriva por parecido con B7</t>
+  </si>
+  <si>
+    <t>calidad "200HV" (G13) → material NO se deriva (deliberatelyUncovered): ni INOX/AC ni sugerencia</t>
   </si>
   <si>
     <t>name</t>
@@ -254,6 +491,12 @@
     <t>nombre "bullone" (IT, no está en §3) → fuera de familia; nombre es solo lectura hoy</t>
   </si>
   <si>
+    <t>nombre "Schraube" (DE) y acabado "verzinkt" (DE) → los dos fuera de tabla; doble candidato de alta en dos vocabularios</t>
+  </si>
+  <si>
+    <t>nombre "parafuso" (PT, no está en §3) → fuera de familia; nombre es solo lectura hoy</t>
+  </si>
+  <si>
     <t>norma</t>
   </si>
   <si>
@@ -263,25 +506,31 @@
     <t>norma "ASME B18.2.2" sin equivalencia DIN→ISO → se conserva tal cual</t>
   </si>
   <si>
+    <t>norma "UNI 5739" (IT) fuera de la tabla DIN→ISO → se conserva; norma es solo lectura hoy</t>
+  </si>
+  <si>
+    <t>norma "BS 3692" (UK) se conserva; calidad "GR R" además no tiene derivación de material → hueco P-3 en la misma fila</t>
+  </si>
+  <si>
     <t>mix</t>
   </si>
   <si>
     <t>ACABADO + MATERIAL</t>
   </si>
   <si>
+    <t>HDG + GR B8M</t>
+  </si>
+  <si>
+    <t>sí (los dos)</t>
+  </si>
+  <si>
+    <t>acabado "HDG" resuelve por tabla Y calidad "GR B8M" pide alta de material → verde y revisión a la vez</t>
+  </si>
+  <si>
     <t>tropicalizado + GR L43</t>
   </si>
   <si>
-    <t>sí (los dos)</t>
-  </si>
-  <si>
     <t>acabado "tropicalizado" (P-12) Y calidad "GR L43" sin material → dos altas, misma fila</t>
-  </si>
-  <si>
-    <t>control</t>
-  </si>
-  <si>
-    <t>—</t>
   </si>
   <si>
     <t>control: nombre, calidad, norma y acabado ya cubiertos → resuelta</t>
@@ -674,7 +923,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -900,28 +1149,28 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
+      <c r="E11">
+        <v>100</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" t="s">
         <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11">
-        <v>200</v>
-      </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -929,16 +1178,16 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E12">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
@@ -947,10 +1196,10 @@
         <v>14</v>
       </c>
       <c r="H12" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="I12" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -958,16 +1207,16 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E13">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="F13" t="s">
         <v>13</v>
@@ -976,10 +1225,10 @@
         <v>14</v>
       </c>
       <c r="H13" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="I13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -987,28 +1236,28 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="E14">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F14" t="s">
         <v>13</v>
       </c>
       <c r="G14" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="H14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="I14" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1016,28 +1265,28 @@
         <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="E15">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="F15" t="s">
         <v>13</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H15" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="I15" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1051,10 +1300,10 @@
         <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E16">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="F16" t="s">
         <v>13</v>
@@ -1063,10 +1312,10 @@
         <v>14</v>
       </c>
       <c r="H16" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="I16" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1074,16 +1323,16 @@
         <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E17">
-        <v>70</v>
+        <v>400</v>
       </c>
       <c r="F17" t="s">
         <v>13</v>
@@ -1092,10 +1341,10 @@
         <v>14</v>
       </c>
       <c r="H17" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I17" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -1103,16 +1352,16 @@
         <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E18">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="F18" t="s">
         <v>13</v>
@@ -1121,10 +1370,10 @@
         <v>14</v>
       </c>
       <c r="H18" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="I18" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1138,10 +1387,10 @@
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="E19">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="F19" t="s">
         <v>13</v>
@@ -1150,10 +1399,10 @@
         <v>14</v>
       </c>
       <c r="H19" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I19" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1161,28 +1410,782 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20">
+        <v>55</v>
+      </c>
+      <c r="F20" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" t="s">
+        <v>24</v>
+      </c>
+      <c r="I20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>17</v>
+      </c>
+      <c r="B21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21">
+        <v>30</v>
+      </c>
+      <c r="F21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>18</v>
+      </c>
+      <c r="B22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22">
+        <v>130</v>
+      </c>
+      <c r="F22" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>19</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23">
+        <v>220</v>
+      </c>
+      <c r="F23" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24">
+        <v>500</v>
+      </c>
+      <c r="F24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>21</v>
+      </c>
+      <c r="B25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25">
+        <v>200</v>
+      </c>
+      <c r="F25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" t="s">
+        <v>67</v>
+      </c>
+      <c r="I25" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>22</v>
+      </c>
+      <c r="B26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" t="s">
+        <v>53</v>
+      </c>
+      <c r="E26">
+        <v>40</v>
+      </c>
+      <c r="F26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" t="s">
+        <v>70</v>
+      </c>
+      <c r="I26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>23</v>
+      </c>
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27">
+        <v>90</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" t="s">
+        <v>74</v>
+      </c>
+      <c r="I27" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>24</v>
+      </c>
+      <c r="B28" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28">
+        <v>35</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" t="s">
+        <v>70</v>
+      </c>
+      <c r="I28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>25</v>
+      </c>
+      <c r="B29" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" t="s">
+        <v>77</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29">
+        <v>70</v>
+      </c>
+      <c r="F29" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" t="s">
+        <v>15</v>
+      </c>
+      <c r="I29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>26</v>
+      </c>
+      <c r="B30" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E30">
+        <v>180</v>
+      </c>
+      <c r="F30" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" t="s">
+        <v>14</v>
+      </c>
+      <c r="H30" t="s">
+        <v>24</v>
+      </c>
+      <c r="I30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>27</v>
+      </c>
+      <c r="B31" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31">
+        <v>300</v>
+      </c>
+      <c r="F31" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I31" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>28</v>
+      </c>
+      <c r="B32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" t="s">
+        <v>82</v>
+      </c>
+      <c r="D32" t="s">
+        <v>83</v>
+      </c>
+      <c r="E32">
+        <v>50</v>
+      </c>
+      <c r="F32" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" t="s">
+        <v>14</v>
+      </c>
+      <c r="H32" t="s">
+        <v>70</v>
+      </c>
+      <c r="I32" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33">
+        <v>20</v>
+      </c>
+      <c r="F33" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" t="s">
+        <v>14</v>
+      </c>
+      <c r="H33" t="s">
+        <v>86</v>
+      </c>
+      <c r="I33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>30</v>
+      </c>
+      <c r="B34" t="s">
+        <v>87</v>
+      </c>
+      <c r="C34" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34">
+        <v>600</v>
+      </c>
+      <c r="F34" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" t="s">
+        <v>14</v>
+      </c>
+      <c r="H34" t="s">
+        <v>90</v>
+      </c>
+      <c r="I34" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>31</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35">
+        <v>50</v>
+      </c>
+      <c r="F35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" t="s">
+        <v>92</v>
+      </c>
+      <c r="H35" t="s">
+        <v>93</v>
+      </c>
+      <c r="I35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>32</v>
+      </c>
+      <c r="B36" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36">
+        <v>40</v>
+      </c>
+      <c r="F36" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" t="s">
+        <v>94</v>
+      </c>
+      <c r="H36" t="s">
+        <v>95</v>
+      </c>
+      <c r="I36" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>33</v>
+      </c>
+      <c r="B37" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" t="s">
+        <v>30</v>
+      </c>
+      <c r="E37">
+        <v>250</v>
+      </c>
+      <c r="F37" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" t="s">
+        <v>96</v>
+      </c>
+      <c r="H37" t="s">
+        <v>15</v>
+      </c>
+      <c r="I37" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" t="s">
+        <v>98</v>
+      </c>
+      <c r="E38">
+        <v>350</v>
+      </c>
+      <c r="F38" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" t="s">
+        <v>99</v>
+      </c>
+      <c r="H38" t="s">
+        <v>15</v>
+      </c>
+      <c r="I38" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>35</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" t="s">
+        <v>100</v>
+      </c>
+      <c r="E39">
+        <v>70</v>
+      </c>
+      <c r="F39" t="s">
+        <v>13</v>
+      </c>
+      <c r="G39" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" t="s">
+        <v>101</v>
+      </c>
+      <c r="I39" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>36</v>
+      </c>
+      <c r="B40" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" t="s">
+        <v>102</v>
+      </c>
+      <c r="E40">
+        <v>70</v>
+      </c>
+      <c r="F40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" t="s">
+        <v>14</v>
+      </c>
+      <c r="H40" t="s">
+        <v>103</v>
+      </c>
+      <c r="I40" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>37</v>
+      </c>
+      <c r="B41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
+        <v>104</v>
+      </c>
+      <c r="E41">
+        <v>95</v>
+      </c>
+      <c r="F41" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" t="s">
+        <v>105</v>
+      </c>
+      <c r="I41" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>38</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" t="s">
+        <v>106</v>
+      </c>
+      <c r="D42" t="s">
+        <v>107</v>
+      </c>
+      <c r="E42">
+        <v>40</v>
+      </c>
+      <c r="F42" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" t="s">
+        <v>14</v>
+      </c>
+      <c r="H42" t="s">
+        <v>108</v>
+      </c>
+      <c r="I42" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>39</v>
+      </c>
+      <c r="B43" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" t="s">
+        <v>82</v>
+      </c>
+      <c r="D43" t="s">
+        <v>110</v>
+      </c>
+      <c r="E43">
+        <v>30</v>
+      </c>
+      <c r="F43" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" t="s">
+        <v>14</v>
+      </c>
+      <c r="H43" t="s">
+        <v>70</v>
+      </c>
+      <c r="I43" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>40</v>
+      </c>
+      <c r="B44" t="s">
+        <v>65</v>
+      </c>
+      <c r="C44" t="s">
+        <v>111</v>
+      </c>
+      <c r="D44" t="s">
+        <v>112</v>
+      </c>
+      <c r="E44">
+        <v>25</v>
+      </c>
+      <c r="F44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" t="s">
+        <v>14</v>
+      </c>
+      <c r="H44" t="s">
+        <v>67</v>
+      </c>
+      <c r="I44" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>41</v>
       </c>
-      <c r="C20" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" t="s">
-        <v>52</v>
-      </c>
-      <c r="E20">
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45">
         <v>100</v>
       </c>
-      <c r="F20" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" t="s">
-        <v>57</v>
-      </c>
-      <c r="I20" t="s">
-        <v>40</v>
+      <c r="F45" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" t="s">
+        <v>14</v>
+      </c>
+      <c r="H45" t="s">
+        <v>15</v>
+      </c>
+      <c r="I45" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>42</v>
+      </c>
+      <c r="B46" t="s">
+        <v>46</v>
+      </c>
+      <c r="C46" t="s">
+        <v>113</v>
+      </c>
+      <c r="D46" t="s">
+        <v>102</v>
+      </c>
+      <c r="E46">
+        <v>100</v>
+      </c>
+      <c r="F46" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" t="s">
+        <v>14</v>
+      </c>
+      <c r="H46" t="s">
+        <v>49</v>
+      </c>
+      <c r="I46" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1193,7 +2196,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1209,19 +2212,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1229,7 +2232,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -1238,10 +2241,10 @@
         <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1249,7 +2252,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -1258,10 +2261,10 @@
         <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1269,7 +2272,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1278,10 +2281,10 @@
         <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="F4" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1289,7 +2292,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -1298,10 +2301,10 @@
         <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1309,7 +2312,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -1318,10 +2321,10 @@
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1329,7 +2332,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -1338,10 +2341,10 @@
         <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1349,19 +2352,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>3</v>
+        <v>128</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>128</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="F8" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1369,19 +2372,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
-        <v>3</v>
+        <v>128</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>128</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1389,19 +2392,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
-        <v>3</v>
+        <v>128</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="F10" t="s">
-        <v>76</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1409,19 +2412,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>127</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>128</v>
       </c>
       <c r="D11" t="s">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1429,19 +2432,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>127</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
+        <v>128</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>128</v>
       </c>
       <c r="E12" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1449,19 +2452,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>80</v>
+        <v>127</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>128</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1469,19 +2472,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>128</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1489,19 +2492,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="E15" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1509,19 +2512,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1529,19 +2532,539 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>120</v>
+      </c>
+      <c r="F17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" t="s">
+        <v>120</v>
+      </c>
+      <c r="F18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" t="s">
+        <v>120</v>
+      </c>
+      <c r="F19" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" t="s">
+        <v>120</v>
+      </c>
+      <c r="F20" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" t="s">
+        <v>120</v>
+      </c>
+      <c r="F21" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>143</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" t="s">
+        <v>120</v>
+      </c>
+      <c r="F22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>143</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" t="s">
+        <v>120</v>
+      </c>
+      <c r="F23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E24" t="s">
+        <v>147</v>
+      </c>
+      <c r="F24" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" t="s">
+        <v>128</v>
+      </c>
+      <c r="E25" t="s">
+        <v>128</v>
+      </c>
+      <c r="F25" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26" t="s">
+        <v>128</v>
+      </c>
+      <c r="F26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" t="s">
+        <v>128</v>
+      </c>
+      <c r="D27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" t="s">
+        <v>128</v>
+      </c>
+      <c r="F27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" t="s">
+        <v>128</v>
+      </c>
+      <c r="D28" t="s">
+        <v>128</v>
+      </c>
+      <c r="E28" t="s">
+        <v>128</v>
+      </c>
+      <c r="F28" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>143</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3</v>
+      </c>
+      <c r="D29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" t="s">
+        <v>120</v>
+      </c>
+      <c r="F29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>143</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D30" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" t="s">
+        <v>120</v>
+      </c>
+      <c r="F30" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+      <c r="D31" t="s">
         <v>88</v>
       </c>
-      <c r="C17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D17" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" t="s">
-        <v>89</v>
-      </c>
-      <c r="F17" t="s">
-        <v>91</v>
+      <c r="E31" t="s">
+        <v>120</v>
+      </c>
+      <c r="F31" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>156</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" t="s">
+        <v>92</v>
+      </c>
+      <c r="E32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" t="s">
+        <v>147</v>
+      </c>
+      <c r="F33" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>156</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" t="s">
+        <v>147</v>
+      </c>
+      <c r="F34" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>156</v>
+      </c>
+      <c r="C35" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" t="s">
+        <v>147</v>
+      </c>
+      <c r="F35" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>101</v>
+      </c>
+      <c r="E36" t="s">
+        <v>147</v>
+      </c>
+      <c r="F36" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>103</v>
+      </c>
+      <c r="E37" t="s">
+        <v>147</v>
+      </c>
+      <c r="F37" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>161</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>105</v>
+      </c>
+      <c r="E38" t="s">
+        <v>147</v>
+      </c>
+      <c r="F38" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>161</v>
+      </c>
+      <c r="C39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" t="s">
+        <v>108</v>
+      </c>
+      <c r="E39" t="s">
+        <v>147</v>
+      </c>
+      <c r="F39" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>166</v>
+      </c>
+      <c r="C40" t="s">
+        <v>167</v>
+      </c>
+      <c r="D40" t="s">
+        <v>168</v>
+      </c>
+      <c r="E40" t="s">
+        <v>169</v>
+      </c>
+      <c r="F40" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>166</v>
+      </c>
+      <c r="C41" t="s">
+        <v>167</v>
+      </c>
+      <c r="D41" t="s">
+        <v>171</v>
+      </c>
+      <c r="E41" t="s">
+        <v>169</v>
+      </c>
+      <c r="F41" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>127</v>
+      </c>
+      <c r="C42" t="s">
+        <v>128</v>
+      </c>
+      <c r="D42" t="s">
+        <v>128</v>
+      </c>
+      <c r="E42" t="s">
+        <v>128</v>
+      </c>
+      <c r="F42" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>127</v>
+      </c>
+      <c r="C43" t="s">
+        <v>128</v>
+      </c>
+      <c r="D43" t="s">
+        <v>128</v>
+      </c>
+      <c r="E43" t="s">
+        <v>128</v>
+      </c>
+      <c r="F43" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>